<commit_message>
UI update; better design
</commit_message>
<xml_diff>
--- a/exports/research_data_master.xlsx
+++ b/exports/research_data_master.xlsx
@@ -33,19 +33,19 @@
     <t>Partner Type</t>
   </si>
   <si>
-    <t>participant_1764874312665</t>
-  </si>
-  <si>
-    <t>msg_1764874329587_rq1ybpltj_0</t>
+    <t>participant_1766278633551</t>
+  </si>
+  <si>
+    <t>msg_1766278791402_udn004g08_0</t>
   </si>
   <si>
     <t>participant</t>
   </si>
   <si>
-    <t>hello</t>
-  </si>
-  <si>
-    <t>2025-12-04T18:52:09.587Z</t>
+    <t>hi</t>
+  </si>
+  <si>
+    <t>2025-12-21T00:59:51.402Z</t>
   </si>
   <si>
     <t>llm</t>
@@ -87,7 +87,7 @@
     <t>Export Date</t>
   </si>
   <si>
-    <t>2025-12-04T18:52:09.592Z</t>
+    <t>2025-12-21T00:59:51.412Z</t>
   </si>
   <si>
     <t>Total Sessions</t>
@@ -636,7 +636,7 @@
         <v>25</v>
       </c>
       <c r="B3">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -644,7 +644,7 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <v>72</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>